<commit_message>
readme file changed to 750 words
</commit_message>
<xml_diff>
--- a/datafiles/sheet.xlsx
+++ b/datafiles/sheet.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andriod\Documents\SearchKeywordBasedOnDayAndSaveInExcel\datafiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E68D6E-87AC-4A69-BB94-5782273285A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D12A94-6E91-4C1E-9C11-7D830A324042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Saturday" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="60">
   <si>
     <t>Longest Option</t>
   </si>
@@ -185,11 +185,54 @@
   <si>
     <t>Shortest Option</t>
   </si>
+  <si>
+    <t>dhaka education board
+Board of Intermediate and Secondary Education, Dhaka · 5 Joynag Rd, Dhaka</t>
+  </si>
+  <si>
+    <t>Dhaka-7</t>
+  </si>
+  <si>
+    <t>Baby Shark
+Song by Pinkfong</t>
+  </si>
+  <si>
+    <t>baby</t>
+  </si>
+  <si>
+    <t>school magazine paragraph</t>
+  </si>
+  <si>
+    <t>Cricket World Cup
+Sports cup</t>
+  </si>
+  <si>
+    <t>pathao courier tracking</t>
+  </si>
+  <si>
+    <t>International League T20
+Cricket league</t>
+  </si>
+  <si>
+    <t>internet speed</t>
+  </si>
+  <si>
+    <t>look change lifestyle salon
+Look Change Lifestyle Saloon · Dhanmondi 9/A, Eastern Elite Center, Meena Bazaar [3rd floor], House no-50. Block-D, Opposite of Ibne Sina, Dhaka</t>
+  </si>
+  <si>
+    <t>hello ai</t>
+  </si>
+  <si>
+    <t>Byeon Woo-seok
+South Korean model and actor</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -538,12 +581,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" customWidth="1"/>
-    <col min="4" max="4" width="76.85546875" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="13.5703125"/>
+    <col min="3" max="3" customWidth="true" width="17.85546875"/>
+    <col min="4" max="4" customWidth="true" width="76.85546875"/>
+    <col min="5" max="5" customWidth="true" width="41.42578125"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -574,10 +617,10 @@
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>28</v>
       </c>
     </row>
@@ -589,10 +632,10 @@
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" t="s" s="0">
         <v>30</v>
       </c>
     </row>
@@ -604,10 +647,10 @@
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" t="s" s="0">
         <v>31</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" t="s" s="0">
         <v>32</v>
       </c>
     </row>
@@ -619,10 +662,10 @@
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" t="s" s="0">
         <v>33</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" t="s" s="0">
         <v>34</v>
       </c>
     </row>
@@ -634,10 +677,10 @@
       <c r="C7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" t="s" s="0">
         <v>36</v>
       </c>
     </row>
@@ -649,10 +692,10 @@
       <c r="C8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" t="s" s="0">
         <v>37</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" t="s" s="0">
         <v>38</v>
       </c>
     </row>
@@ -664,10 +707,10 @@
       <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" t="s" s="0">
         <v>39</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" t="s" s="0">
         <v>40</v>
       </c>
     </row>
@@ -679,10 +722,10 @@
       <c r="C10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" t="s" s="0">
         <v>41</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" t="s" s="0">
         <v>42</v>
       </c>
     </row>
@@ -694,10 +737,10 @@
       <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" t="s" s="0">
         <v>43</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" t="s" s="0">
         <v>44</v>
       </c>
     </row>
@@ -709,10 +752,10 @@
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" t="s" s="0">
         <v>46</v>
       </c>
     </row>
@@ -1719,12 +1762,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="29.42578125" customWidth="1"/>
-    <col min="5" max="5" width="33.28515625" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="14.140625"/>
+    <col min="3" max="3" customWidth="true" width="17.5703125"/>
+    <col min="4" max="4" customWidth="true" width="29.42578125"/>
+    <col min="5" max="5" customWidth="true" width="33.28515625"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2864,12 +2907,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="4" width="28.5703125" customWidth="1"/>
-    <col min="5" max="5" width="31.85546875" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="13.42578125"/>
+    <col min="3" max="3" customWidth="true" width="8.7109375"/>
+    <col min="4" max="4" customWidth="true" width="28.5703125"/>
+    <col min="5" max="5" customWidth="true" width="31.85546875"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4009,12 +4052,12 @@
   <dimension ref="A2:F1001"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="30.85546875" customWidth="1"/>
-    <col min="5" max="5" width="39.5703125" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="16.140625"/>
+    <col min="3" max="3" customWidth="true" width="16.42578125"/>
+    <col min="4" max="4" customWidth="true" width="30.85546875"/>
+    <col min="5" max="5" customWidth="true" width="39.5703125"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -5146,12 +5189,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" customWidth="1"/>
-    <col min="5" max="5" width="29.5703125" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="13.28515625"/>
+    <col min="3" max="3" customWidth="true" width="20.85546875"/>
+    <col min="4" max="4" customWidth="true" width="33.7109375"/>
+    <col min="5" max="5" customWidth="true" width="29.5703125"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5182,6 +5225,12 @@
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D3" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>49</v>
+      </c>
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -5192,8 +5241,12 @@
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="D4" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>30</v>
+      </c>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -5204,8 +5257,12 @@
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
+      <c r="D5" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>51</v>
+      </c>
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -5216,8 +5273,12 @@
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="D6" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>34</v>
+      </c>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -5228,8 +5289,12 @@
       <c r="C7" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="D7" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>36</v>
+      </c>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -5240,8 +5305,12 @@
       <c r="C8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="D8" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>24</v>
+      </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -5252,8 +5321,12 @@
       <c r="C9" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="D9" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>56</v>
+      </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -5264,8 +5337,12 @@
       <c r="C10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="D10" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>42</v>
+      </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -5276,8 +5353,12 @@
       <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="D11" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>58</v>
+      </c>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -5288,8 +5369,12 @@
       <c r="C12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="D12" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="E12" t="s">
+        <v>46</v>
+      </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -6291,12 +6376,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="33" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="8.7109375"/>
+    <col min="2" max="2" customWidth="true" width="19.140625"/>
+    <col min="3" max="3" customWidth="true" width="17.0"/>
+    <col min="4" max="4" customWidth="true" width="33.0"/>
+    <col min="5" max="5" customWidth="true" width="28.85546875"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7436,12 +7521,12 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" customWidth="1"/>
-    <col min="5" max="5" width="36.28515625" customWidth="1"/>
-    <col min="6" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.28515625"/>
+    <col min="2" max="2" customWidth="true" width="15.0"/>
+    <col min="3" max="3" customWidth="true" width="16.7109375"/>
+    <col min="4" max="4" customWidth="true" width="31.140625"/>
+    <col min="5" max="5" customWidth="true" width="36.28515625"/>
+    <col min="6" max="26" customWidth="true" width="8.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>